<commit_message>
Backlog al dia: sprints 06-08 cerrados, HU-50 hecha y H-16 de UX cargada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backlog_CooperApp_2026.xlsx
+++ b/Backlog_CooperApp_2026.xlsx
@@ -28,7 +28,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cambios vs. original" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Product Backlog'!$A$4:$I$423</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Product Backlog'!$A$4:$I$424</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -928,7 +928,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Período: 21/09 al 27/09    |    Estado: En curso</t>
+          <t>Período: 21/09 al 27/09    |    Estado: Cerrado</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1451,7 +1451,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Período: 28/09 al 04/10    |    Estado: En curso</t>
+          <t>Período: 28/09 al 04/10    |    Estado: Cerrado</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2189,7 +2189,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Período: 05/10 al 11/10    |    Estado: Planificado</t>
+          <t>Período: 05/10 al 11/10    |    Estado: En curso</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3268,10 +3268,14 @@
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D49" s="23" t="inlineStr"/>
+      <c r="D49" s="23" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
       <c r="E49" s="24" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
     </row>
@@ -3287,10 +3291,14 @@
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr"/>
-      <c r="D50" s="14" t="inlineStr"/>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
       <c r="E50" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
     </row>
@@ -3306,10 +3314,14 @@
         </is>
       </c>
       <c r="C51" s="16" t="inlineStr"/>
-      <c r="D51" s="16" t="inlineStr"/>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
       <c r="E51" s="17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
     </row>
@@ -3325,10 +3337,14 @@
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr"/>
-      <c r="D52" s="14" t="inlineStr"/>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
       <c r="E52" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3422,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Período: 12/10 al 18/10    |    Estado: Planificado</t>
+          <t>Período: 12/10 al 18/10    |    Estado: En curso</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -4663,7 +4679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4927,434 +4943,453 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="23" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>T-64.5</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Decidir con usuarios si el resultado por servicio vive en Movimientos o en Reportes</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr"/>
+      <c r="D16" s="14" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>HU-87</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>Como tesorero quiero cargar un movimiento en menos pasos para no contestar tres preguntas encadenadas.</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D16" s="23" t="inlineStr"/>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="D17" s="23" t="inlineStr"/>
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>T-87.1</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Reemplazar los tres desplegables encadenados por uno solo</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr"/>
-      <c r="D17" s="14" t="inlineStr"/>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr"/>
+      <c r="D18" s="14" t="inlineStr"/>
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>T-87.2</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">     Permitir corregir un movimiento anulado sin escribirlo de nuevo</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr"/>
-      <c r="D18" s="16" t="inlineStr"/>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr"/>
+      <c r="D19" s="16" t="inlineStr"/>
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="23" t="inlineStr">
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>HU-88</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Como usuario quiero que las pantallas vacías me digan por dónde empezar en vez de culpar a un filtro que no toqué.</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D19" s="23" t="inlineStr"/>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="D20" s="23" t="inlineStr"/>
+      <c r="E20" s="24" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>T-88.1</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Separar el listado vacío del listado filtrado en los cuatro listados</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr"/>
-      <c r="D20" s="14" t="inlineStr"/>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr"/>
+      <c r="D21" s="14" t="inlineStr"/>
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>T-88.2</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">     Agregar un bloque de primeros pasos al panel de una empresa nueva</t>
         </is>
       </c>
-      <c r="C21" s="16" t="inlineStr"/>
-      <c r="D21" s="16" t="inlineStr"/>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr"/>
+      <c r="D22" s="16" t="inlineStr"/>
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>T-88.3</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Poner 'Sin acceso' en los indicadores que el rol no puede ver</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr"/>
-      <c r="D22" s="14" t="inlineStr"/>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr"/>
+      <c r="D23" s="14" t="inlineStr"/>
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="23" t="inlineStr">
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>HU-65</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>Como usuario quiero usar todo el sistema desde el celular para trabajar donde estoy.</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D23" s="23" t="inlineStr"/>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="D24" s="23" t="inlineStr"/>
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>T-65.1</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Colapsar los filtros detrás de un botón en las pantallas de listado</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr"/>
-      <c r="D24" s="14" t="inlineStr"/>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr"/>
+      <c r="D25" s="14" t="inlineStr"/>
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>T-65.2</t>
         </is>
       </c>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">     Revisar las pantallas de los módulos nuevos en ancho de celular</t>
         </is>
       </c>
-      <c r="C25" s="16" t="inlineStr"/>
-      <c r="D25" s="16" t="inlineStr"/>
-      <c r="E25" s="17" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr"/>
+      <c r="D26" s="16" t="inlineStr"/>
+      <c r="E26" s="17" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>T-65.3</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Validar en Chrome y en un segundo navegador</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr"/>
-      <c r="D26" s="14" t="inlineStr"/>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr"/>
+      <c r="D27" s="14" t="inlineStr"/>
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>T-65.4</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">     Validar en un celular real</t>
         </is>
       </c>
-      <c r="C27" s="16" t="inlineStr"/>
-      <c r="D27" s="16" t="inlineStr"/>
-      <c r="E27" s="17" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr"/>
+      <c r="D28" s="16" t="inlineStr"/>
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="23" t="inlineStr">
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>HU-66</t>
         </is>
       </c>
-      <c r="B28" s="23" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>Como equipo quiero dejar el proyecto documentado para poder continuarlo el año próximo.</t>
         </is>
       </c>
-      <c r="C28" s="23" t="inlineStr">
+      <c r="C29" s="23" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D28" s="23" t="inlineStr"/>
-      <c r="E28" s="24" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr"/>
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>T-66.1</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Escribir el README con las instrucciones de instalación</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr"/>
-      <c r="D29" s="14" t="inlineStr"/>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr"/>
+      <c r="D30" s="14" t="inlineStr"/>
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>T-66.2</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">     Escribir el manual de usuario básico</t>
         </is>
       </c>
-      <c r="C30" s="16" t="inlineStr"/>
-      <c r="D30" s="16" t="inlineStr"/>
-      <c r="E30" s="17" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr"/>
+      <c r="D31" s="16" t="inlineStr"/>
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>T-66.3</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Documentar el modelo de datos</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr"/>
-      <c r="D31" s="14" t="inlineStr"/>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr"/>
+      <c r="D32" s="14" t="inlineStr"/>
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>T-66.4</t>
         </is>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">     Documentar el diseño de los módulos que quedaron sin implementar</t>
         </is>
       </c>
-      <c r="C32" s="16" t="inlineStr"/>
-      <c r="D32" s="16" t="inlineStr"/>
-      <c r="E32" s="17" t="inlineStr">
+      <c r="C33" s="16" t="inlineStr"/>
+      <c r="D33" s="16" t="inlineStr"/>
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>HU-67</t>
         </is>
       </c>
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B34" s="23" t="inlineStr">
         <is>
           <t>Como equipo quiero probar el sistema completo para entregar una versión estable.</t>
         </is>
       </c>
-      <c r="C33" s="23" t="inlineStr">
+      <c r="C34" s="23" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D33" s="23" t="inlineStr"/>
-      <c r="E33" s="24" t="inlineStr">
+      <c r="D34" s="23" t="inlineStr"/>
+      <c r="E34" s="24" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>T-67.1</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Ejecutar la batería de pruebas de punta a punta</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr"/>
-      <c r="D34" s="14" t="inlineStr"/>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr"/>
+      <c r="D35" s="14" t="inlineStr"/>
+      <c r="E35" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>T-67.2</t>
         </is>
       </c>
-      <c r="B35" s="16" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">     Corregir los errores detectados</t>
         </is>
       </c>
-      <c r="C35" s="16" t="inlineStr"/>
-      <c r="D35" s="16" t="inlineStr"/>
-      <c r="E35" s="17" t="inlineStr">
+      <c r="C36" s="16" t="inlineStr"/>
+      <c r="D36" s="16" t="inlineStr"/>
+      <c r="E36" s="17" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>T-67.3</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">     Unificar la carga del encabezado en un archivo compartido</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr"/>
-      <c r="D36" s="14" t="inlineStr"/>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr"/>
+      <c r="D37" s="14" t="inlineStr"/>
+      <c r="E37" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="C38" s="19" t="inlineStr">
+    <row r="39">
+      <c r="C39" s="19" t="inlineStr">
         <is>
           <t>AVANCE DEL SPRINT (tareas terminadas)</t>
         </is>
       </c>
-      <c r="D38" s="20" t="n"/>
-      <c r="E38" s="20">
-        <f>TEXT(SUMPRODUCT((LEFT(A6:A36,2)="T-")*(E6:E36="Hecho"))/SUMPRODUCT((LEFT(A6:A36,2)="T-")*1),"0%")</f>
+      <c r="D39" s="20" t="n"/>
+      <c r="E39" s="20">
+        <f>TEXT(SUMPRODUCT((LEFT(A6:A37,2)="T-")*(E6:E37="Hecho"))/SUMPRODUCT((LEFT(A6:A37,2)="T-")*1),"0%")</f>
         <v/>
       </c>
     </row>
@@ -5364,7 +5399,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E36">
+  <conditionalFormatting sqref="E6:E37">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Hecho"</formula>
     </cfRule>
@@ -5379,10 +5414,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E6:E36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E6:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,En curso,En revisión,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="D6:D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D6:D37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aguilera Maximiliano,Hoyos Franco,Delipetro Ezequiel,Achille Nahuel,Equipo"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6695,7 +6730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I423"/>
+  <dimension ref="A1:I424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19953,10 +19988,14 @@
       </c>
       <c r="H336" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I336" s="12" t="inlineStr"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I336" s="12" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="14" t="inlineStr">
@@ -19988,10 +20027,14 @@
       </c>
       <c r="H337" s="14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I337" s="14" t="inlineStr"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I337" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="16" t="inlineStr">
@@ -20023,10 +20066,14 @@
       </c>
       <c r="H338" s="16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I338" s="16" t="inlineStr"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I338" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="14" t="inlineStr">
@@ -20058,10 +20105,14 @@
       </c>
       <c r="H339" s="14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I339" s="14" t="inlineStr"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I339" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
     </row>
     <row r="340" ht="16" customHeight="1">
       <c r="A340" s="12" t="inlineStr">
@@ -20507,2757 +20558,2792 @@
       </c>
       <c r="I351" s="16" t="inlineStr"/>
     </row>
-    <row r="352" ht="26" customHeight="1">
-      <c r="A352" s="12" t="inlineStr">
+    <row r="352">
+      <c r="A352" s="14" t="inlineStr">
+        <is>
+          <t>T-64.5</t>
+        </is>
+      </c>
+      <c r="B352" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C352" s="14" t="inlineStr"/>
+      <c r="D352" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Decidir con usuarios si el resultado por servicio vive en Movimientos o en Reportes</t>
+        </is>
+      </c>
+      <c r="E352" s="15" t="inlineStr"/>
+      <c r="F352" s="15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G352" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 13</t>
+        </is>
+      </c>
+      <c r="H352" s="14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I352" s="14" t="inlineStr"/>
+    </row>
+    <row r="353" ht="26" customHeight="1">
+      <c r="A353" s="12" t="inlineStr">
         <is>
           <t>HU-87</t>
         </is>
       </c>
-      <c r="B352" s="12" t="inlineStr">
+      <c r="B353" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C352" s="12" t="inlineStr">
+      <c r="C353" s="12" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D352" s="12" t="inlineStr">
+      <c r="D353" s="12" t="inlineStr">
         <is>
           <t>Como tesorero quiero cargar un movimiento en menos pasos para no contestar tres preguntas encadenadas.</t>
         </is>
       </c>
-      <c r="E352" s="13" t="inlineStr">
+      <c r="E353" s="13" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F352" s="13" t="inlineStr">
+      <c r="F353" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G352" s="13" t="inlineStr">
+      <c r="G353" s="13" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H352" s="12" t="inlineStr">
+      <c r="H353" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I352" s="12" t="inlineStr"/>
-    </row>
-    <row r="353">
-      <c r="A353" s="14" t="inlineStr">
+      <c r="I353" s="12" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="14" t="inlineStr">
         <is>
           <t>T-87.1</t>
         </is>
       </c>
-      <c r="B353" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C353" s="14" t="inlineStr"/>
-      <c r="D353" s="14" t="inlineStr">
+      <c r="B354" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C354" s="14" t="inlineStr"/>
+      <c r="D354" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Reemplazar los tres desplegables encadenados por uno solo</t>
         </is>
       </c>
-      <c r="E353" s="15" t="inlineStr"/>
-      <c r="F353" s="15" t="inlineStr">
+      <c r="E354" s="15" t="inlineStr"/>
+      <c r="F354" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G353" s="15" t="inlineStr">
+      <c r="G354" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H353" s="14" t="inlineStr">
+      <c r="H354" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I353" s="14" t="inlineStr"/>
-    </row>
-    <row r="354">
-      <c r="A354" s="16" t="inlineStr">
+      <c r="I354" s="14" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="16" t="inlineStr">
         <is>
           <t>T-87.2</t>
         </is>
       </c>
-      <c r="B354" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C354" s="16" t="inlineStr"/>
-      <c r="D354" s="16" t="inlineStr">
+      <c r="B355" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C355" s="16" t="inlineStr"/>
+      <c r="D355" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Permitir corregir un movimiento anulado sin escribirlo de nuevo</t>
         </is>
       </c>
-      <c r="E354" s="17" t="inlineStr"/>
-      <c r="F354" s="17" t="inlineStr">
+      <c r="E355" s="17" t="inlineStr"/>
+      <c r="F355" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G354" s="17" t="inlineStr">
+      <c r="G355" s="17" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H354" s="16" t="inlineStr">
+      <c r="H355" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I354" s="16" t="inlineStr"/>
-    </row>
-    <row r="355" ht="26" customHeight="1">
-      <c r="A355" s="12" t="inlineStr">
+      <c r="I355" s="16" t="inlineStr"/>
+    </row>
+    <row r="356" ht="26" customHeight="1">
+      <c r="A356" s="12" t="inlineStr">
         <is>
           <t>HU-88</t>
         </is>
       </c>
-      <c r="B355" s="12" t="inlineStr">
+      <c r="B356" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C355" s="12" t="inlineStr">
+      <c r="C356" s="12" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D355" s="12" t="inlineStr">
+      <c r="D356" s="12" t="inlineStr">
         <is>
           <t>Como usuario quiero que las pantallas vacías me digan por dónde empezar en vez de culpar a un filtro que no toqué.</t>
         </is>
       </c>
-      <c r="E355" s="13" t="inlineStr">
+      <c r="E356" s="13" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F355" s="13" t="inlineStr">
+      <c r="F356" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G355" s="13" t="inlineStr">
+      <c r="G356" s="13" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H355" s="12" t="inlineStr">
+      <c r="H356" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I355" s="12" t="inlineStr"/>
-    </row>
-    <row r="356">
-      <c r="A356" s="14" t="inlineStr">
+      <c r="I356" s="12" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="14" t="inlineStr">
         <is>
           <t>T-88.1</t>
         </is>
       </c>
-      <c r="B356" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C356" s="14" t="inlineStr"/>
-      <c r="D356" s="14" t="inlineStr">
+      <c r="B357" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C357" s="14" t="inlineStr"/>
+      <c r="D357" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Separar el listado vacío del listado filtrado en los cuatro listados</t>
         </is>
       </c>
-      <c r="E356" s="15" t="inlineStr"/>
-      <c r="F356" s="15" t="inlineStr">
+      <c r="E357" s="15" t="inlineStr"/>
+      <c r="F357" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G356" s="15" t="inlineStr">
+      <c r="G357" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H356" s="14" t="inlineStr">
+      <c r="H357" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I356" s="14" t="inlineStr"/>
-    </row>
-    <row r="357">
-      <c r="A357" s="16" t="inlineStr">
+      <c r="I357" s="14" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="16" t="inlineStr">
         <is>
           <t>T-88.2</t>
         </is>
       </c>
-      <c r="B357" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C357" s="16" t="inlineStr"/>
-      <c r="D357" s="16" t="inlineStr">
+      <c r="B358" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C358" s="16" t="inlineStr"/>
+      <c r="D358" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Agregar un bloque de primeros pasos al panel de una empresa nueva</t>
         </is>
       </c>
-      <c r="E357" s="17" t="inlineStr"/>
-      <c r="F357" s="17" t="inlineStr">
+      <c r="E358" s="17" t="inlineStr"/>
+      <c r="F358" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G357" s="17" t="inlineStr">
+      <c r="G358" s="17" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H357" s="16" t="inlineStr">
+      <c r="H358" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I357" s="16" t="inlineStr"/>
-    </row>
-    <row r="358">
-      <c r="A358" s="14" t="inlineStr">
+      <c r="I358" s="16" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="14" t="inlineStr">
         <is>
           <t>T-88.3</t>
         </is>
       </c>
-      <c r="B358" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C358" s="14" t="inlineStr"/>
-      <c r="D358" s="14" t="inlineStr">
+      <c r="B359" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C359" s="14" t="inlineStr"/>
+      <c r="D359" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Poner 'Sin acceso' en los indicadores que el rol no puede ver</t>
         </is>
       </c>
-      <c r="E358" s="15" t="inlineStr"/>
-      <c r="F358" s="15" t="inlineStr">
+      <c r="E359" s="15" t="inlineStr"/>
+      <c r="F359" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G358" s="15" t="inlineStr">
+      <c r="G359" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H358" s="14" t="inlineStr">
+      <c r="H359" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I358" s="14" t="inlineStr"/>
-    </row>
-    <row r="359" ht="16" customHeight="1">
-      <c r="A359" s="12" t="inlineStr">
+      <c r="I359" s="14" t="inlineStr"/>
+    </row>
+    <row r="360" ht="16" customHeight="1">
+      <c r="A360" s="12" t="inlineStr">
         <is>
           <t>HU-65</t>
         </is>
       </c>
-      <c r="B359" s="12" t="inlineStr">
+      <c r="B360" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C359" s="12" t="inlineStr">
+      <c r="C360" s="12" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D359" s="12" t="inlineStr">
+      <c r="D360" s="12" t="inlineStr">
         <is>
           <t>Como usuario quiero usar todo el sistema desde el celular para trabajar donde estoy.</t>
         </is>
       </c>
-      <c r="E359" s="13" t="inlineStr">
+      <c r="E360" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F359" s="13" t="inlineStr">
+      <c r="F360" s="13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G359" s="13" t="inlineStr">
+      <c r="G360" s="13" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H359" s="12" t="inlineStr">
+      <c r="H360" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I359" s="12" t="inlineStr"/>
-    </row>
-    <row r="360">
-      <c r="A360" s="14" t="inlineStr">
+      <c r="I360" s="12" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="14" t="inlineStr">
         <is>
           <t>T-65.1</t>
         </is>
       </c>
-      <c r="B360" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C360" s="14" t="inlineStr"/>
-      <c r="D360" s="14" t="inlineStr">
+      <c r="B361" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C361" s="14" t="inlineStr"/>
+      <c r="D361" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Colapsar los filtros detrás de un botón en las pantallas de listado</t>
         </is>
       </c>
-      <c r="E360" s="15" t="inlineStr"/>
-      <c r="F360" s="15" t="inlineStr">
+      <c r="E361" s="15" t="inlineStr"/>
+      <c r="F361" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G360" s="15" t="inlineStr">
+      <c r="G361" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H360" s="14" t="inlineStr">
+      <c r="H361" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I360" s="14" t="inlineStr"/>
-    </row>
-    <row r="361">
-      <c r="A361" s="16" t="inlineStr">
+      <c r="I361" s="14" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="16" t="inlineStr">
         <is>
           <t>T-65.2</t>
         </is>
       </c>
-      <c r="B361" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C361" s="16" t="inlineStr"/>
-      <c r="D361" s="16" t="inlineStr">
+      <c r="B362" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C362" s="16" t="inlineStr"/>
+      <c r="D362" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Revisar las pantallas de los módulos nuevos en ancho de celular</t>
         </is>
       </c>
-      <c r="E361" s="17" t="inlineStr"/>
-      <c r="F361" s="17" t="inlineStr">
+      <c r="E362" s="17" t="inlineStr"/>
+      <c r="F362" s="17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G361" s="17" t="inlineStr">
+      <c r="G362" s="17" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H361" s="16" t="inlineStr">
+      <c r="H362" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I361" s="16" t="inlineStr"/>
-    </row>
-    <row r="362">
-      <c r="A362" s="14" t="inlineStr">
+      <c r="I362" s="16" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="14" t="inlineStr">
         <is>
           <t>T-65.3</t>
         </is>
       </c>
-      <c r="B362" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C362" s="14" t="inlineStr"/>
-      <c r="D362" s="14" t="inlineStr">
+      <c r="B363" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C363" s="14" t="inlineStr"/>
+      <c r="D363" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Validar en Chrome y en un segundo navegador</t>
         </is>
       </c>
-      <c r="E362" s="15" t="inlineStr"/>
-      <c r="F362" s="15" t="inlineStr">
+      <c r="E363" s="15" t="inlineStr"/>
+      <c r="F363" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G362" s="15" t="inlineStr">
+      <c r="G363" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H362" s="14" t="inlineStr">
+      <c r="H363" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I362" s="14" t="inlineStr"/>
-    </row>
-    <row r="363">
-      <c r="A363" s="16" t="inlineStr">
+      <c r="I363" s="14" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="16" t="inlineStr">
         <is>
           <t>T-65.4</t>
         </is>
       </c>
-      <c r="B363" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C363" s="16" t="inlineStr"/>
-      <c r="D363" s="16" t="inlineStr">
+      <c r="B364" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C364" s="16" t="inlineStr"/>
+      <c r="D364" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Validar en un celular real</t>
         </is>
       </c>
-      <c r="E363" s="17" t="inlineStr"/>
-      <c r="F363" s="17" t="inlineStr">
+      <c r="E364" s="17" t="inlineStr"/>
+      <c r="F364" s="17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G363" s="17" t="inlineStr">
+      <c r="G364" s="17" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H363" s="16" t="inlineStr">
+      <c r="H364" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I363" s="16" t="inlineStr"/>
-    </row>
-    <row r="364" ht="16" customHeight="1">
-      <c r="A364" s="12" t="inlineStr">
+      <c r="I364" s="16" t="inlineStr"/>
+    </row>
+    <row r="365" ht="16" customHeight="1">
+      <c r="A365" s="12" t="inlineStr">
         <is>
           <t>HU-66</t>
         </is>
       </c>
-      <c r="B364" s="12" t="inlineStr">
+      <c r="B365" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C364" s="12" t="inlineStr">
+      <c r="C365" s="12" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D364" s="12" t="inlineStr">
+      <c r="D365" s="12" t="inlineStr">
         <is>
           <t>Como equipo quiero dejar el proyecto documentado para poder continuarlo el año próximo.</t>
         </is>
       </c>
-      <c r="E364" s="13" t="inlineStr">
+      <c r="E365" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F364" s="13" t="inlineStr">
+      <c r="F365" s="13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G364" s="13" t="inlineStr">
+      <c r="G365" s="13" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H364" s="12" t="inlineStr">
+      <c r="H365" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I364" s="12" t="inlineStr"/>
-    </row>
-    <row r="365">
-      <c r="A365" s="14" t="inlineStr">
+      <c r="I365" s="12" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="14" t="inlineStr">
         <is>
           <t>T-66.1</t>
         </is>
       </c>
-      <c r="B365" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C365" s="14" t="inlineStr"/>
-      <c r="D365" s="14" t="inlineStr">
+      <c r="B366" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C366" s="14" t="inlineStr"/>
+      <c r="D366" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Escribir el README con las instrucciones de instalación</t>
         </is>
       </c>
-      <c r="E365" s="15" t="inlineStr"/>
-      <c r="F365" s="15" t="inlineStr">
+      <c r="E366" s="15" t="inlineStr"/>
+      <c r="F366" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G365" s="15" t="inlineStr">
+      <c r="G366" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H365" s="14" t="inlineStr">
+      <c r="H366" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I365" s="14" t="inlineStr"/>
-    </row>
-    <row r="366">
-      <c r="A366" s="16" t="inlineStr">
+      <c r="I366" s="14" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="16" t="inlineStr">
         <is>
           <t>T-66.2</t>
         </is>
       </c>
-      <c r="B366" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C366" s="16" t="inlineStr"/>
-      <c r="D366" s="16" t="inlineStr">
+      <c r="B367" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C367" s="16" t="inlineStr"/>
+      <c r="D367" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Escribir el manual de usuario básico</t>
         </is>
       </c>
-      <c r="E366" s="17" t="inlineStr"/>
-      <c r="F366" s="17" t="inlineStr">
+      <c r="E367" s="17" t="inlineStr"/>
+      <c r="F367" s="17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G366" s="17" t="inlineStr">
+      <c r="G367" s="17" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H366" s="16" t="inlineStr">
+      <c r="H367" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I366" s="16" t="inlineStr"/>
-    </row>
-    <row r="367">
-      <c r="A367" s="14" t="inlineStr">
+      <c r="I367" s="16" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="14" t="inlineStr">
         <is>
           <t>T-66.3</t>
         </is>
       </c>
-      <c r="B367" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C367" s="14" t="inlineStr"/>
-      <c r="D367" s="14" t="inlineStr">
+      <c r="B368" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C368" s="14" t="inlineStr"/>
+      <c r="D368" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Documentar el modelo de datos</t>
         </is>
       </c>
-      <c r="E367" s="15" t="inlineStr"/>
-      <c r="F367" s="15" t="inlineStr">
+      <c r="E368" s="15" t="inlineStr"/>
+      <c r="F368" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G367" s="15" t="inlineStr">
+      <c r="G368" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H367" s="14" t="inlineStr">
+      <c r="H368" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I367" s="14" t="inlineStr"/>
-    </row>
-    <row r="368">
-      <c r="A368" s="16" t="inlineStr">
+      <c r="I368" s="14" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="16" t="inlineStr">
         <is>
           <t>T-66.4</t>
         </is>
       </c>
-      <c r="B368" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C368" s="16" t="inlineStr"/>
-      <c r="D368" s="16" t="inlineStr">
+      <c r="B369" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C369" s="16" t="inlineStr"/>
+      <c r="D369" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Documentar el diseño de los módulos que quedaron sin implementar</t>
         </is>
       </c>
-      <c r="E368" s="17" t="inlineStr"/>
-      <c r="F368" s="17" t="inlineStr">
+      <c r="E369" s="17" t="inlineStr"/>
+      <c r="F369" s="17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G368" s="17" t="inlineStr">
+      <c r="G369" s="17" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H368" s="16" t="inlineStr">
+      <c r="H369" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I368" s="16" t="inlineStr"/>
-    </row>
-    <row r="369" ht="16" customHeight="1">
-      <c r="A369" s="12" t="inlineStr">
+      <c r="I369" s="16" t="inlineStr"/>
+    </row>
+    <row r="370" ht="16" customHeight="1">
+      <c r="A370" s="12" t="inlineStr">
         <is>
           <t>HU-67</t>
         </is>
       </c>
-      <c r="B369" s="12" t="inlineStr">
+      <c r="B370" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C369" s="12" t="inlineStr">
+      <c r="C370" s="12" t="inlineStr">
         <is>
           <t>Calidad, UX y Documentación</t>
         </is>
       </c>
-      <c r="D369" s="12" t="inlineStr">
+      <c r="D370" s="12" t="inlineStr">
         <is>
           <t>Como equipo quiero probar el sistema completo para entregar una versión estable.</t>
         </is>
       </c>
-      <c r="E369" s="13" t="inlineStr">
+      <c r="E370" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F369" s="13" t="inlineStr">
+      <c r="F370" s="13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G369" s="13" t="inlineStr">
+      <c r="G370" s="13" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H369" s="12" t="inlineStr">
+      <c r="H370" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I369" s="12" t="inlineStr"/>
-    </row>
-    <row r="370">
-      <c r="A370" s="14" t="inlineStr">
+      <c r="I370" s="12" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="14" t="inlineStr">
         <is>
           <t>T-67.1</t>
         </is>
       </c>
-      <c r="B370" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C370" s="14" t="inlineStr"/>
-      <c r="D370" s="14" t="inlineStr">
+      <c r="B371" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C371" s="14" t="inlineStr"/>
+      <c r="D371" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Ejecutar la batería de pruebas de punta a punta</t>
         </is>
       </c>
-      <c r="E370" s="15" t="inlineStr"/>
-      <c r="F370" s="15" t="inlineStr">
+      <c r="E371" s="15" t="inlineStr"/>
+      <c r="F371" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G370" s="15" t="inlineStr">
+      <c r="G371" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H370" s="14" t="inlineStr">
+      <c r="H371" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I370" s="14" t="inlineStr"/>
-    </row>
-    <row r="371">
-      <c r="A371" s="16" t="inlineStr">
+      <c r="I371" s="14" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="16" t="inlineStr">
         <is>
           <t>T-67.2</t>
         </is>
       </c>
-      <c r="B371" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C371" s="16" t="inlineStr"/>
-      <c r="D371" s="16" t="inlineStr">
+      <c r="B372" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C372" s="16" t="inlineStr"/>
+      <c r="D372" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Corregir los errores detectados</t>
         </is>
       </c>
-      <c r="E371" s="17" t="inlineStr"/>
-      <c r="F371" s="17" t="inlineStr">
+      <c r="E372" s="17" t="inlineStr"/>
+      <c r="F372" s="17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G371" s="17" t="inlineStr">
+      <c r="G372" s="17" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H371" s="16" t="inlineStr">
+      <c r="H372" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I371" s="16" t="inlineStr"/>
-    </row>
-    <row r="372">
-      <c r="A372" s="14" t="inlineStr">
+      <c r="I372" s="16" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="14" t="inlineStr">
         <is>
           <t>T-67.3</t>
         </is>
       </c>
-      <c r="B372" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C372" s="14" t="inlineStr"/>
-      <c r="D372" s="14" t="inlineStr">
+      <c r="B373" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C373" s="14" t="inlineStr"/>
+      <c r="D373" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Unificar la carga del encabezado en un archivo compartido</t>
         </is>
       </c>
-      <c r="E372" s="15" t="inlineStr"/>
-      <c r="F372" s="15" t="inlineStr">
+      <c r="E373" s="15" t="inlineStr"/>
+      <c r="F373" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G372" s="15" t="inlineStr">
+      <c r="G373" s="15" t="inlineStr">
         <is>
           <t>Sprint 13</t>
         </is>
       </c>
-      <c r="H372" s="14" t="inlineStr">
+      <c r="H373" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I372" s="14" t="inlineStr"/>
-    </row>
-    <row r="373" ht="20" customHeight="1">
-      <c r="A373" s="9" t="inlineStr">
+      <c r="I373" s="14" t="inlineStr"/>
+    </row>
+    <row r="374" ht="20" customHeight="1">
+      <c r="A374" s="9" t="inlineStr">
         <is>
           <t>E11</t>
         </is>
       </c>
-      <c r="B373" s="9" t="inlineStr">
+      <c r="B374" s="9" t="inlineStr">
         <is>
           <t>Épica</t>
         </is>
       </c>
-      <c r="C373" s="9" t="inlineStr">
+      <c r="C374" s="9" t="inlineStr">
         <is>
           <t>Chat y Notificaciones</t>
         </is>
       </c>
-      <c r="D373" s="9" t="inlineStr">
+      <c r="D374" s="9" t="inlineStr">
         <is>
           <t>Mensajería entre empresas (posterior al MVP)</t>
         </is>
       </c>
-      <c r="E373" s="10" t="inlineStr">
+      <c r="E374" s="10" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="F373" s="11" t="n"/>
-      <c r="G373" s="11" t="n"/>
-      <c r="H373" s="11" t="n"/>
-      <c r="I373" s="11" t="n"/>
-    </row>
-    <row r="374" ht="16" customHeight="1">
-      <c r="A374" s="12" t="inlineStr">
+      <c r="F374" s="11" t="n"/>
+      <c r="G374" s="11" t="n"/>
+      <c r="H374" s="11" t="n"/>
+      <c r="I374" s="11" t="n"/>
+    </row>
+    <row r="375" ht="16" customHeight="1">
+      <c r="A375" s="12" t="inlineStr">
         <is>
           <t>HU-73</t>
         </is>
       </c>
-      <c r="B374" s="12" t="inlineStr">
+      <c r="B375" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C374" s="12" t="inlineStr">
+      <c r="C375" s="12" t="inlineStr">
         <is>
           <t>Chat y Notificaciones</t>
         </is>
       </c>
-      <c r="D374" s="12" t="inlineStr">
+      <c r="D375" s="12" t="inlineStr">
         <is>
           <t>Como empresa quiero chatear con otra empresa para coordinar una articulación.</t>
         </is>
       </c>
-      <c r="E374" s="13" t="inlineStr">
+      <c r="E375" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="F374" s="13" t="inlineStr">
+      <c r="F375" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G374" s="13" t="inlineStr">
+      <c r="G375" s="13" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H374" s="12" t="inlineStr">
+      <c r="H375" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I374" s="12" t="inlineStr"/>
-    </row>
-    <row r="375">
-      <c r="A375" s="14" t="inlineStr">
+      <c r="I375" s="12" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="14" t="inlineStr">
         <is>
           <t>T-73.1</t>
         </is>
       </c>
-      <c r="B375" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C375" s="14" t="inlineStr"/>
-      <c r="D375" s="14" t="inlineStr">
+      <c r="B376" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C376" s="14" t="inlineStr"/>
+      <c r="D376" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Diseñar la pantalla de chat</t>
         </is>
       </c>
-      <c r="E375" s="15" t="inlineStr"/>
-      <c r="F375" s="15" t="inlineStr">
+      <c r="E376" s="15" t="inlineStr"/>
+      <c r="F376" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G375" s="15" t="inlineStr">
+      <c r="G376" s="15" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H375" s="14" t="inlineStr">
+      <c r="H376" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I375" s="14" t="inlineStr"/>
-    </row>
-    <row r="376">
-      <c r="A376" s="16" t="inlineStr">
+      <c r="I376" s="14" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="16" t="inlineStr">
         <is>
           <t>T-73.2</t>
         </is>
       </c>
-      <c r="B376" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C376" s="16" t="inlineStr"/>
-      <c r="D376" s="16" t="inlineStr">
+      <c r="B377" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C377" s="16" t="inlineStr"/>
+      <c r="D377" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar el envío y la recepción de mensajes</t>
         </is>
       </c>
-      <c r="E376" s="17" t="inlineStr"/>
-      <c r="F376" s="17" t="inlineStr">
+      <c r="E377" s="17" t="inlineStr"/>
+      <c r="F377" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G376" s="17" t="inlineStr">
+      <c r="G377" s="17" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H376" s="16" t="inlineStr">
+      <c r="H377" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I376" s="16" t="inlineStr"/>
-    </row>
-    <row r="377">
-      <c r="A377" s="14" t="inlineStr">
+      <c r="I377" s="16" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="14" t="inlineStr">
         <is>
           <t>T-73.3</t>
         </is>
       </c>
-      <c r="B377" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C377" s="14" t="inlineStr"/>
-      <c r="D377" s="14" t="inlineStr">
+      <c r="B378" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C378" s="14" t="inlineStr"/>
+      <c r="D378" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Agregar notificaciones de mensaje nuevo</t>
         </is>
       </c>
-      <c r="E377" s="15" t="inlineStr"/>
-      <c r="F377" s="15" t="inlineStr">
+      <c r="E378" s="15" t="inlineStr"/>
+      <c r="F378" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G377" s="15" t="inlineStr">
+      <c r="G378" s="15" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H377" s="14" t="inlineStr">
+      <c r="H378" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I377" s="14" t="inlineStr"/>
-    </row>
-    <row r="378" ht="20" customHeight="1">
-      <c r="A378" s="9" t="inlineStr">
+      <c r="I378" s="14" t="inlineStr"/>
+    </row>
+    <row r="379" ht="20" customHeight="1">
+      <c r="A379" s="9" t="inlineStr">
         <is>
           <t>E12</t>
         </is>
       </c>
-      <c r="B378" s="9" t="inlineStr">
+      <c r="B379" s="9" t="inlineStr">
         <is>
           <t>Épica</t>
         </is>
       </c>
-      <c r="C378" s="9" t="inlineStr">
+      <c r="C379" s="9" t="inlineStr">
         <is>
           <t>Configuración de Módulos</t>
         </is>
       </c>
-      <c r="D378" s="9" t="inlineStr">
+      <c r="D379" s="9" t="inlineStr">
         <is>
           <t>Cada empresa activa sólo los módulos que usa</t>
         </is>
       </c>
-      <c r="E378" s="10" t="inlineStr">
+      <c r="E379" s="10" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F378" s="11" t="n"/>
-      <c r="G378" s="11" t="n"/>
-      <c r="H378" s="11" t="n"/>
-      <c r="I378" s="11" t="n"/>
-    </row>
-    <row r="379" ht="26" customHeight="1">
-      <c r="A379" s="12" t="inlineStr">
+      <c r="F379" s="11" t="n"/>
+      <c r="G379" s="11" t="n"/>
+      <c r="H379" s="11" t="n"/>
+      <c r="I379" s="11" t="n"/>
+    </row>
+    <row r="380" ht="26" customHeight="1">
+      <c r="A380" s="12" t="inlineStr">
         <is>
           <t>HU-34</t>
         </is>
       </c>
-      <c r="B379" s="12" t="inlineStr">
+      <c r="B380" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C379" s="12" t="inlineStr">
+      <c r="C380" s="12" t="inlineStr">
         <is>
           <t>Configuración de Módulos</t>
         </is>
       </c>
-      <c r="D379" s="12" t="inlineStr">
+      <c r="D380" s="12" t="inlineStr">
         <is>
           <t>Como administrador de la empresa quiero activar sólo los módulos que mi empresa usa para no ver funciones que no necesito.</t>
         </is>
       </c>
-      <c r="E379" s="13" t="inlineStr">
+      <c r="E380" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F379" s="13" t="inlineStr">
+      <c r="F380" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G379" s="13" t="inlineStr">
+      <c r="G380" s="13" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H379" s="12" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I379" s="12" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" s="14" t="inlineStr">
+      <c r="H380" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I380" s="12" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="14" t="inlineStr">
         <is>
           <t>T-34.1</t>
         </is>
       </c>
-      <c r="B380" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C380" s="14" t="inlineStr"/>
-      <c r="D380" s="14" t="inlineStr">
+      <c r="B381" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C381" s="14" t="inlineStr"/>
+      <c r="D381" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Crear la tabla de módulos activos por empresa</t>
         </is>
       </c>
-      <c r="E380" s="15" t="inlineStr"/>
-      <c r="F380" s="15" t="inlineStr">
+      <c r="E381" s="15" t="inlineStr"/>
+      <c r="F381" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G380" s="15" t="inlineStr">
+      <c r="G381" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H380" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I380" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" s="16" t="inlineStr">
+      <c r="H381" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I381" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="16" t="inlineStr">
         <is>
           <t>T-34.2</t>
         </is>
       </c>
-      <c r="B381" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C381" s="16" t="inlineStr"/>
-      <c r="D381" s="16" t="inlineStr">
+      <c r="B382" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C382" s="16" t="inlineStr"/>
+      <c r="D382" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Definir el conjunto de módulos disponibles</t>
         </is>
       </c>
-      <c r="E381" s="17" t="inlineStr"/>
-      <c r="F381" s="17" t="inlineStr">
+      <c r="E382" s="17" t="inlineStr"/>
+      <c r="F382" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G381" s="17" t="inlineStr">
+      <c r="G382" s="17" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H381" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I381" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" s="14" t="inlineStr">
+      <c r="H382" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I382" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="14" t="inlineStr">
         <is>
           <t>T-34.3</t>
         </is>
       </c>
-      <c r="B382" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C382" s="14" t="inlineStr"/>
-      <c r="D382" s="14" t="inlineStr">
+      <c r="B383" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C383" s="14" t="inlineStr"/>
+      <c r="D383" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar los endpoints de consulta y actualización</t>
         </is>
       </c>
-      <c r="E382" s="15" t="inlineStr"/>
-      <c r="F382" s="15" t="inlineStr">
+      <c r="E383" s="15" t="inlineStr"/>
+      <c r="F383" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G382" s="15" t="inlineStr">
+      <c r="G383" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H382" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I382" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" s="16" t="inlineStr">
+      <c r="H383" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I383" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="16" t="inlineStr">
         <is>
           <t>T-34.4</t>
         </is>
       </c>
-      <c r="B383" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C383" s="16" t="inlineStr"/>
-      <c r="D383" s="16" t="inlineStr">
+      <c r="B384" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C384" s="16" t="inlineStr"/>
+      <c r="D384" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Diseñar la pantalla de configuración de módulos</t>
         </is>
       </c>
-      <c r="E383" s="17" t="inlineStr"/>
-      <c r="F383" s="17" t="inlineStr">
+      <c r="E384" s="17" t="inlineStr"/>
+      <c r="F384" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G383" s="17" t="inlineStr">
+      <c r="G384" s="17" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H383" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I383" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" s="14" t="inlineStr">
+      <c r="H384" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I384" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="14" t="inlineStr">
         <is>
           <t>T-34.5</t>
         </is>
       </c>
-      <c r="B384" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C384" s="14" t="inlineStr"/>
-      <c r="D384" s="14" t="inlineStr">
+      <c r="B385" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C385" s="14" t="inlineStr"/>
+      <c r="D385" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Mostrar en el menú sólo los módulos activos</t>
         </is>
       </c>
-      <c r="E384" s="15" t="inlineStr"/>
-      <c r="F384" s="15" t="inlineStr">
+      <c r="E385" s="15" t="inlineStr"/>
+      <c r="F385" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G384" s="15" t="inlineStr">
+      <c r="G385" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H384" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I384" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="385" ht="26" customHeight="1">
-      <c r="A385" s="12" t="inlineStr">
+      <c r="H385" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I385" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="386" ht="26" customHeight="1">
+      <c r="A386" s="12" t="inlineStr">
         <is>
           <t>HU-35</t>
         </is>
       </c>
-      <c r="B385" s="12" t="inlineStr">
+      <c r="B386" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C385" s="12" t="inlineStr">
+      <c r="C386" s="12" t="inlineStr">
         <is>
           <t>Configuración de Módulos</t>
         </is>
       </c>
-      <c r="D385" s="12" t="inlineStr">
+      <c r="D386" s="12" t="inlineStr">
         <is>
           <t>Como sistema quiero rechazar los pedidos a módulos desactivados para que no se pueda entrar por fuera del menú.</t>
         </is>
       </c>
-      <c r="E385" s="13" t="inlineStr">
+      <c r="E386" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F385" s="13" t="inlineStr">
+      <c r="F386" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G385" s="13" t="inlineStr">
+      <c r="G386" s="13" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H385" s="12" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I385" s="12" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" s="14" t="inlineStr">
+      <c r="H386" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I386" s="12" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="14" t="inlineStr">
         <is>
           <t>T-35.1</t>
         </is>
       </c>
-      <c r="B386" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C386" s="14" t="inlineStr"/>
-      <c r="D386" s="14" t="inlineStr">
+      <c r="B387" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C387" s="14" t="inlineStr"/>
+      <c r="D387" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar el middleware de módulo activo</t>
         </is>
       </c>
-      <c r="E386" s="15" t="inlineStr"/>
-      <c r="F386" s="15" t="inlineStr">
+      <c r="E387" s="15" t="inlineStr"/>
+      <c r="F387" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G386" s="15" t="inlineStr">
+      <c r="G387" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H386" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I386" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="387">
-      <c r="A387" s="16" t="inlineStr">
+      <c r="H387" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I387" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="16" t="inlineStr">
         <is>
           <t>T-35.2</t>
         </is>
       </c>
-      <c r="B387" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C387" s="16" t="inlineStr"/>
-      <c r="D387" s="16" t="inlineStr">
+      <c r="B388" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C388" s="16" t="inlineStr"/>
+      <c r="D388" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Aplicarlo a las rutas de movimientos y categorías</t>
         </is>
       </c>
-      <c r="E387" s="17" t="inlineStr"/>
-      <c r="F387" s="17" t="inlineStr">
+      <c r="E388" s="17" t="inlineStr"/>
+      <c r="F388" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G387" s="17" t="inlineStr">
+      <c r="G388" s="17" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H387" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I387" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="388">
-      <c r="A388" s="14" t="inlineStr">
+      <c r="H388" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I388" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="14" t="inlineStr">
         <is>
           <t>T-35.3</t>
         </is>
       </c>
-      <c r="B388" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C388" s="14" t="inlineStr"/>
-      <c r="D388" s="14" t="inlineStr">
+      <c r="B389" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C389" s="14" t="inlineStr"/>
+      <c r="D389" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Mostrar en pantalla un aviso claro cuando el módulo está apagado</t>
         </is>
       </c>
-      <c r="E388" s="15" t="inlineStr"/>
-      <c r="F388" s="15" t="inlineStr">
+      <c r="E389" s="15" t="inlineStr"/>
+      <c r="F389" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G388" s="15" t="inlineStr">
+      <c r="G389" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H388" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I388" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="389">
-      <c r="A389" s="16" t="inlineStr">
+      <c r="H389" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I389" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="16" t="inlineStr">
         <is>
           <t>T-35.4</t>
         </is>
       </c>
-      <c r="B389" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C389" s="16" t="inlineStr"/>
-      <c r="D389" s="16" t="inlineStr">
+      <c r="B390" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C390" s="16" t="inlineStr"/>
+      <c r="D390" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Distinguir el aviso de módulo apagado del de falta de permiso</t>
         </is>
       </c>
-      <c r="E389" s="17" t="inlineStr"/>
-      <c r="F389" s="17" t="inlineStr">
+      <c r="E390" s="17" t="inlineStr"/>
+      <c r="F390" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G389" s="17" t="inlineStr">
+      <c r="G390" s="17" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H389" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I389" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="390">
-      <c r="A390" s="14" t="inlineStr">
+      <c r="H390" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I390" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="14" t="inlineStr">
         <is>
           <t>T-35.5</t>
         </is>
       </c>
-      <c r="B390" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C390" s="14" t="inlineStr"/>
-      <c r="D390" s="14" t="inlineStr">
+      <c r="B391" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C391" s="14" t="inlineStr"/>
+      <c r="D391" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Probar el acceso con el módulo apagado</t>
         </is>
       </c>
-      <c r="E390" s="15" t="inlineStr"/>
-      <c r="F390" s="15" t="inlineStr">
+      <c r="E391" s="15" t="inlineStr"/>
+      <c r="F391" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G390" s="15" t="inlineStr">
+      <c r="G391" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H390" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I390" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="391" ht="26" customHeight="1">
-      <c r="A391" s="12" t="inlineStr">
+      <c r="H391" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I391" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="26" customHeight="1">
+      <c r="A392" s="12" t="inlineStr">
         <is>
           <t>HU-36</t>
         </is>
       </c>
-      <c r="B391" s="12" t="inlineStr">
+      <c r="B392" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C391" s="12" t="inlineStr">
+      <c r="C392" s="12" t="inlineStr">
         <is>
           <t>Configuración de Módulos</t>
         </is>
       </c>
-      <c r="D391" s="12" t="inlineStr">
+      <c r="D392" s="12" t="inlineStr">
         <is>
           <t>Como empresa nueva quiero empezar con una configuración razonable para no tener que definir todo antes de usar el sistema.</t>
         </is>
       </c>
-      <c r="E391" s="13" t="inlineStr">
+      <c r="E392" s="13" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F391" s="13" t="inlineStr">
+      <c r="F392" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G391" s="13" t="inlineStr">
+      <c r="G392" s="13" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H391" s="12" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I391" s="12" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="392">
-      <c r="A392" s="14" t="inlineStr">
+      <c r="H392" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I392" s="12" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="14" t="inlineStr">
         <is>
           <t>T-36.1</t>
         </is>
       </c>
-      <c r="B392" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C392" s="14" t="inlineStr"/>
-      <c r="D392" s="14" t="inlineStr">
+      <c r="B393" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C393" s="14" t="inlineStr"/>
+      <c r="D393" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Definir el conjunto de módulos y categorías iniciales</t>
         </is>
       </c>
-      <c r="E392" s="15" t="inlineStr"/>
-      <c r="F392" s="15" t="inlineStr">
+      <c r="E393" s="15" t="inlineStr"/>
+      <c r="F393" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G392" s="15" t="inlineStr">
+      <c r="G393" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H392" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I392" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="393">
-      <c r="A393" s="16" t="inlineStr">
+      <c r="H393" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I393" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="16" t="inlineStr">
         <is>
           <t>T-36.2</t>
         </is>
       </c>
-      <c r="B393" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C393" s="16" t="inlineStr"/>
-      <c r="D393" s="16" t="inlineStr">
+      <c r="B394" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C394" s="16" t="inlineStr"/>
+      <c r="D394" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar la carga automática al aprobar la empresa</t>
         </is>
       </c>
-      <c r="E393" s="17" t="inlineStr"/>
-      <c r="F393" s="17" t="inlineStr">
+      <c r="E394" s="17" t="inlineStr"/>
+      <c r="F394" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G393" s="17" t="inlineStr">
+      <c r="G394" s="17" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H393" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I393" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="394">
-      <c r="A394" s="14" t="inlineStr">
+      <c r="H394" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I394" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="14" t="inlineStr">
         <is>
           <t>T-36.3</t>
         </is>
       </c>
-      <c r="B394" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C394" s="14" t="inlineStr"/>
-      <c r="D394" s="14" t="inlineStr">
+      <c r="B395" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C395" s="14" t="inlineStr"/>
+      <c r="D395" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Dejar la configuración escrita en la base, no deducida del catálogo</t>
         </is>
       </c>
-      <c r="E394" s="15" t="inlineStr"/>
-      <c r="F394" s="15" t="inlineStr">
+      <c r="E395" s="15" t="inlineStr"/>
+      <c r="F395" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G394" s="15" t="inlineStr">
+      <c r="G395" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H394" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I394" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="395">
-      <c r="A395" s="16" t="inlineStr">
+      <c r="H395" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I395" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="16" t="inlineStr">
         <is>
           <t>T-36.4</t>
         </is>
       </c>
-      <c r="B395" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C395" s="16" t="inlineStr"/>
-      <c r="D395" s="16" t="inlineStr">
+      <c r="B396" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C396" s="16" t="inlineStr"/>
+      <c r="D396" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Evitar que una segunda aprobación duplique o pise lo ya configurado</t>
         </is>
       </c>
-      <c r="E395" s="17" t="inlineStr"/>
-      <c r="F395" s="17" t="inlineStr">
+      <c r="E396" s="17" t="inlineStr"/>
+      <c r="F396" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G395" s="17" t="inlineStr">
+      <c r="G396" s="17" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H395" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I395" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="396">
-      <c r="A396" s="14" t="inlineStr">
+      <c r="H396" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I396" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="14" t="inlineStr">
         <is>
           <t>T-36.5</t>
         </is>
       </c>
-      <c r="B396" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C396" s="14" t="inlineStr"/>
-      <c r="D396" s="14" t="inlineStr">
+      <c r="B397" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C397" s="14" t="inlineStr"/>
+      <c r="D397" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Probar el alta de una empresa nueva de punta a punta</t>
         </is>
       </c>
-      <c r="E396" s="15" t="inlineStr"/>
-      <c r="F396" s="15" t="inlineStr">
+      <c r="E397" s="15" t="inlineStr"/>
+      <c r="F397" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G396" s="15" t="inlineStr">
+      <c r="G397" s="15" t="inlineStr">
         <is>
           <t>Sprint 06</t>
         </is>
       </c>
-      <c r="H396" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I396" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="397" ht="20" customHeight="1">
-      <c r="A397" s="9" t="inlineStr">
+      <c r="H397" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I397" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="398" ht="20" customHeight="1">
+      <c r="A398" s="9" t="inlineStr">
         <is>
           <t>E13</t>
         </is>
       </c>
-      <c r="B397" s="9" t="inlineStr">
+      <c r="B398" s="9" t="inlineStr">
         <is>
           <t>Épica</t>
         </is>
       </c>
-      <c r="C397" s="9" t="inlineStr">
+      <c r="C398" s="9" t="inlineStr">
         <is>
           <t>Servicios</t>
         </is>
       </c>
-      <c r="D397" s="9" t="inlineStr">
+      <c r="D398" s="9" t="inlineStr">
         <is>
           <t>Catálogo de servicios que generan ingreso o egreso</t>
         </is>
       </c>
-      <c r="E397" s="10" t="inlineStr">
+      <c r="E398" s="10" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F397" s="11" t="n"/>
-      <c r="G397" s="11" t="n"/>
-      <c r="H397" s="11" t="n"/>
-      <c r="I397" s="11" t="n"/>
-    </row>
-    <row r="398" ht="26" customHeight="1">
-      <c r="A398" s="12" t="inlineStr">
+      <c r="F398" s="11" t="n"/>
+      <c r="G398" s="11" t="n"/>
+      <c r="H398" s="11" t="n"/>
+      <c r="I398" s="11" t="n"/>
+    </row>
+    <row r="399" ht="26" customHeight="1">
+      <c r="A399" s="12" t="inlineStr">
         <is>
           <t>HU-47</t>
         </is>
       </c>
-      <c r="B398" s="12" t="inlineStr">
+      <c r="B399" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C398" s="12" t="inlineStr">
+      <c r="C399" s="12" t="inlineStr">
         <is>
           <t>Servicios</t>
         </is>
       </c>
-      <c r="D398" s="12" t="inlineStr">
+      <c r="D399" s="12" t="inlineStr">
         <is>
           <t>Como administrador quiero cargar los servicios que presta o contrata mi empresa para registrarlos igual que los productos.</t>
         </is>
       </c>
-      <c r="E398" s="13" t="inlineStr">
+      <c r="E399" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F398" s="13" t="inlineStr">
+      <c r="F399" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G398" s="13" t="inlineStr">
+      <c r="G399" s="13" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H398" s="12" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I398" s="12" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="399">
-      <c r="A399" s="14" t="inlineStr">
+      <c r="H399" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I399" s="12" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="14" t="inlineStr">
         <is>
           <t>T-47.1</t>
         </is>
       </c>
-      <c r="B399" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C399" s="14" t="inlineStr"/>
-      <c r="D399" s="14" t="inlineStr">
+      <c r="B400" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C400" s="14" t="inlineStr"/>
+      <c r="D400" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Reutilizar el modelo de productos agregando la distinción de servicio</t>
         </is>
       </c>
-      <c r="E399" s="15" t="inlineStr"/>
-      <c r="F399" s="15" t="inlineStr">
+      <c r="E400" s="15" t="inlineStr"/>
+      <c r="F400" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G399" s="15" t="inlineStr">
+      <c r="G400" s="15" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H399" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I399" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="400">
-      <c r="A400" s="16" t="inlineStr">
+      <c r="H400" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I400" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="16" t="inlineStr">
         <is>
           <t>T-47.2</t>
         </is>
       </c>
-      <c r="B400" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C400" s="16" t="inlineStr"/>
-      <c r="D400" s="16" t="inlineStr">
+      <c r="B401" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C401" s="16" t="inlineStr"/>
+      <c r="D401" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar el alta, la edición y la baja lógica</t>
         </is>
       </c>
-      <c r="E400" s="17" t="inlineStr"/>
-      <c r="F400" s="17" t="inlineStr">
+      <c r="E401" s="17" t="inlineStr"/>
+      <c r="F401" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G400" s="17" t="inlineStr">
+      <c r="G401" s="17" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H400" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I400" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="401">
-      <c r="A401" s="14" t="inlineStr">
+      <c r="H401" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I401" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="14" t="inlineStr">
         <is>
           <t>T-47.3</t>
         </is>
       </c>
-      <c r="B401" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C401" s="14" t="inlineStr"/>
-      <c r="D401" s="14" t="inlineStr">
+      <c r="B402" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C402" s="14" t="inlineStr"/>
+      <c r="D402" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Diseñar la pantalla de servicios</t>
         </is>
       </c>
-      <c r="E401" s="15" t="inlineStr"/>
-      <c r="F401" s="15" t="inlineStr">
+      <c r="E402" s="15" t="inlineStr"/>
+      <c r="F402" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G401" s="15" t="inlineStr">
+      <c r="G402" s="15" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H401" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I401" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="402">
-      <c r="A402" s="16" t="inlineStr">
+      <c r="H402" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I402" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="16" t="inlineStr">
         <is>
           <t>T-47.4</t>
         </is>
       </c>
-      <c r="B402" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C402" s="16" t="inlineStr"/>
-      <c r="D402" s="16" t="inlineStr">
+      <c r="B403" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C403" s="16" t="inlineStr"/>
+      <c r="D403" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Verificar que los servicios no lleven existencias</t>
         </is>
       </c>
-      <c r="E402" s="17" t="inlineStr"/>
-      <c r="F402" s="17" t="inlineStr">
+      <c r="E403" s="17" t="inlineStr"/>
+      <c r="F403" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G402" s="17" t="inlineStr">
+      <c r="G403" s="17" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H402" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I402" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="403" ht="26" customHeight="1">
-      <c r="A403" s="12" t="inlineStr">
+      <c r="H403" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I403" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="404" ht="26" customHeight="1">
+      <c r="A404" s="12" t="inlineStr">
         <is>
           <t>HU-48</t>
         </is>
       </c>
-      <c r="B403" s="12" t="inlineStr">
+      <c r="B404" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C403" s="12" t="inlineStr">
+      <c r="C404" s="12" t="inlineStr">
         <is>
           <t>Servicios</t>
         </is>
       </c>
-      <c r="D403" s="12" t="inlineStr">
+      <c r="D404" s="12" t="inlineStr">
         <is>
           <t>Como tesorero quiero vincular un movimiento de dinero con un servicio para saber de dónde viene cada ingreso o egreso.</t>
         </is>
       </c>
-      <c r="E403" s="13" t="inlineStr">
+      <c r="E404" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F403" s="13" t="inlineStr">
+      <c r="F404" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G403" s="13" t="inlineStr">
+      <c r="G404" s="13" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H403" s="12" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I403" s="12" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="404">
-      <c r="A404" s="14" t="inlineStr">
+      <c r="H404" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I404" s="12" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="14" t="inlineStr">
         <is>
           <t>T-48.1</t>
         </is>
       </c>
-      <c r="B404" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C404" s="14" t="inlineStr"/>
-      <c r="D404" s="14" t="inlineStr">
+      <c r="B405" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C405" s="14" t="inlineStr"/>
+      <c r="D405" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Vincular el movimiento económico con el servicio</t>
         </is>
       </c>
-      <c r="E404" s="15" t="inlineStr"/>
-      <c r="F404" s="15" t="inlineStr">
+      <c r="E405" s="15" t="inlineStr"/>
+      <c r="F405" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G404" s="15" t="inlineStr">
+      <c r="G405" s="15" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H404" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I404" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="405">
-      <c r="A405" s="16" t="inlineStr">
+      <c r="H405" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I405" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="16" t="inlineStr">
         <is>
           <t>T-48.2</t>
         </is>
       </c>
-      <c r="B405" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C405" s="16" t="inlineStr"/>
-      <c r="D405" s="16" t="inlineStr">
+      <c r="B406" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C406" s="16" t="inlineStr"/>
+      <c r="D406" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Agregar el servicio al formulario de movimiento</t>
         </is>
       </c>
-      <c r="E405" s="17" t="inlineStr"/>
-      <c r="F405" s="17" t="inlineStr">
+      <c r="E406" s="17" t="inlineStr"/>
+      <c r="F406" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G405" s="17" t="inlineStr">
+      <c r="G406" s="17" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H405" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I405" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="406">
-      <c r="A406" s="14" t="inlineStr">
+      <c r="H406" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I406" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="14" t="inlineStr">
         <is>
           <t>T-48.3</t>
         </is>
       </c>
-      <c r="B406" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C406" s="14" t="inlineStr"/>
-      <c r="D406" s="14" t="inlineStr">
+      <c r="B407" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C407" s="14" t="inlineStr"/>
+      <c r="D407" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Agregar el filtro por servicio en el listado</t>
         </is>
       </c>
-      <c r="E406" s="15" t="inlineStr"/>
-      <c r="F406" s="15" t="inlineStr">
+      <c r="E407" s="15" t="inlineStr"/>
+      <c r="F407" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G406" s="15" t="inlineStr">
+      <c r="G407" s="15" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H406" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I406" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="407" ht="16" customHeight="1">
-      <c r="A407" s="12" t="inlineStr">
+      <c r="H407" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I407" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="408" ht="16" customHeight="1">
+      <c r="A408" s="12" t="inlineStr">
         <is>
           <t>HU-49</t>
         </is>
       </c>
-      <c r="B407" s="12" t="inlineStr">
+      <c r="B408" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C407" s="12" t="inlineStr">
+      <c r="C408" s="12" t="inlineStr">
         <is>
           <t>Servicios</t>
         </is>
       </c>
-      <c r="D407" s="12" t="inlineStr">
+      <c r="D408" s="12" t="inlineStr">
         <is>
           <t>Como empresa quiero ver cuánto me deja cada servicio para saber cuáles conviene sostener.</t>
         </is>
       </c>
-      <c r="E407" s="13" t="inlineStr">
+      <c r="E408" s="13" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F407" s="13" t="inlineStr">
+      <c r="F408" s="13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G407" s="13" t="inlineStr">
+      <c r="G408" s="13" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H407" s="12" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I407" s="12" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="408">
-      <c r="A408" s="14" t="inlineStr">
+      <c r="H408" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I408" s="12" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="14" t="inlineStr">
         <is>
           <t>T-49.1</t>
         </is>
       </c>
-      <c r="B408" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C408" s="14" t="inlineStr"/>
-      <c r="D408" s="14" t="inlineStr">
+      <c r="B409" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C409" s="14" t="inlineStr"/>
+      <c r="D409" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar la consulta agrupada por servicio</t>
         </is>
       </c>
-      <c r="E408" s="15" t="inlineStr"/>
-      <c r="F408" s="15" t="inlineStr">
+      <c r="E409" s="15" t="inlineStr"/>
+      <c r="F409" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G408" s="15" t="inlineStr">
+      <c r="G409" s="15" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H408" s="14" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I408" s="14" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="409">
-      <c r="A409" s="16" t="inlineStr">
+      <c r="H409" s="14" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I409" s="14" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="16" t="inlineStr">
         <is>
           <t>T-49.2</t>
         </is>
       </c>
-      <c r="B409" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C409" s="16" t="inlineStr"/>
-      <c r="D409" s="16" t="inlineStr">
+      <c r="B410" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C410" s="16" t="inlineStr"/>
+      <c r="D410" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Diseñar la visualización del resumen</t>
         </is>
       </c>
-      <c r="E409" s="17" t="inlineStr"/>
-      <c r="F409" s="17" t="inlineStr">
+      <c r="E410" s="17" t="inlineStr"/>
+      <c r="F410" s="17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G409" s="17" t="inlineStr">
+      <c r="G410" s="17" t="inlineStr">
         <is>
           <t>Sprint 09</t>
         </is>
       </c>
-      <c r="H409" s="16" t="inlineStr">
-        <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="I409" s="16" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="410" ht="20" customHeight="1">
-      <c r="A410" s="9" t="inlineStr">
+      <c r="H410" s="16" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I410" s="16" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="411" ht="20" customHeight="1">
+      <c r="A411" s="9" t="inlineStr">
         <is>
           <t>E14</t>
         </is>
       </c>
-      <c r="B410" s="9" t="inlineStr">
+      <c r="B411" s="9" t="inlineStr">
         <is>
           <t>Épica</t>
         </is>
       </c>
-      <c r="C410" s="9" t="inlineStr">
+      <c r="C411" s="9" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="D410" s="9" t="inlineStr">
+      <c r="D411" s="9" t="inlineStr">
         <is>
           <t>Vacaciones, licencias y documentación del personal (backlog futuro)</t>
         </is>
       </c>
-      <c r="E410" s="10" t="inlineStr">
+      <c r="E411" s="10" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="F410" s="11" t="n"/>
-      <c r="G410" s="11" t="n"/>
-      <c r="H410" s="11" t="n"/>
-      <c r="I410" s="11" t="n"/>
-    </row>
-    <row r="411" ht="16" customHeight="1">
-      <c r="A411" s="12" t="inlineStr">
+      <c r="F411" s="11" t="n"/>
+      <c r="G411" s="11" t="n"/>
+      <c r="H411" s="11" t="n"/>
+      <c r="I411" s="11" t="n"/>
+    </row>
+    <row r="412" ht="16" customHeight="1">
+      <c r="A412" s="12" t="inlineStr">
         <is>
           <t>HU-68</t>
         </is>
       </c>
-      <c r="B411" s="12" t="inlineStr">
+      <c r="B412" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C411" s="12" t="inlineStr">
+      <c r="C412" s="12" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="D411" s="12" t="inlineStr">
+      <c r="D412" s="12" t="inlineStr">
         <is>
           <t>Como empleado quiero solicitar días de vacaciones para gestionarlos sin papeles.</t>
         </is>
       </c>
-      <c r="E411" s="13" t="inlineStr">
+      <c r="E412" s="13" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F411" s="13" t="inlineStr">
+      <c r="F412" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G411" s="13" t="inlineStr">
+      <c r="G412" s="13" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H411" s="12" t="inlineStr">
+      <c r="H412" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I411" s="12" t="inlineStr"/>
-    </row>
-    <row r="412">
-      <c r="A412" s="14" t="inlineStr">
+      <c r="I412" s="12" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="14" t="inlineStr">
         <is>
           <t>T-68.1</t>
         </is>
       </c>
-      <c r="B412" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C412" s="14" t="inlineStr"/>
-      <c r="D412" s="14" t="inlineStr">
+      <c r="B413" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C413" s="14" t="inlineStr"/>
+      <c r="D413" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Diseñar el modelo de licencias y saldo de días</t>
         </is>
       </c>
-      <c r="E412" s="15" t="inlineStr"/>
-      <c r="F412" s="15" t="inlineStr">
+      <c r="E413" s="15" t="inlineStr"/>
+      <c r="F413" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G412" s="15" t="inlineStr">
+      <c r="G413" s="15" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H412" s="14" t="inlineStr">
+      <c r="H413" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I412" s="14" t="inlineStr"/>
-    </row>
-    <row r="413">
-      <c r="A413" s="16" t="inlineStr">
+      <c r="I413" s="14" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" s="16" t="inlineStr">
         <is>
           <t>T-68.2</t>
         </is>
       </c>
-      <c r="B413" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C413" s="16" t="inlineStr"/>
-      <c r="D413" s="16" t="inlineStr">
+      <c r="B414" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C414" s="16" t="inlineStr"/>
+      <c r="D414" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar el circuito de solicitud y aprobación</t>
         </is>
       </c>
-      <c r="E413" s="17" t="inlineStr"/>
-      <c r="F413" s="17" t="inlineStr">
+      <c r="E414" s="17" t="inlineStr"/>
+      <c r="F414" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G413" s="17" t="inlineStr">
+      <c r="G414" s="17" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H413" s="16" t="inlineStr">
+      <c r="H414" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I413" s="16" t="inlineStr"/>
-    </row>
-    <row r="414">
-      <c r="A414" s="14" t="inlineStr">
+      <c r="I414" s="16" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" s="14" t="inlineStr">
         <is>
           <t>T-68.3</t>
         </is>
       </c>
-      <c r="B414" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C414" s="14" t="inlineStr"/>
-      <c r="D414" s="14" t="inlineStr">
+      <c r="B415" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C415" s="14" t="inlineStr"/>
+      <c r="D415" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Diseñar las pantallas de solicitud y de bandeja del responsable</t>
         </is>
       </c>
-      <c r="E414" s="15" t="inlineStr"/>
-      <c r="F414" s="15" t="inlineStr">
+      <c r="E415" s="15" t="inlineStr"/>
+      <c r="F415" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G414" s="15" t="inlineStr">
+      <c r="G415" s="15" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H414" s="14" t="inlineStr">
+      <c r="H415" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I414" s="14" t="inlineStr"/>
-    </row>
-    <row r="415">
-      <c r="A415" s="16" t="inlineStr">
+      <c r="I415" s="14" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" s="16" t="inlineStr">
         <is>
           <t>T-68.4</t>
         </is>
       </c>
-      <c r="B415" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C415" s="16" t="inlineStr"/>
-      <c r="D415" s="16" t="inlineStr">
+      <c r="B416" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C416" s="16" t="inlineStr"/>
+      <c r="D416" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar el cálculo del saldo de días</t>
         </is>
       </c>
-      <c r="E415" s="17" t="inlineStr"/>
-      <c r="F415" s="17" t="inlineStr">
+      <c r="E416" s="17" t="inlineStr"/>
+      <c r="F416" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G415" s="17" t="inlineStr">
+      <c r="G416" s="17" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H415" s="16" t="inlineStr">
+      <c r="H416" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I415" s="16" t="inlineStr"/>
-    </row>
-    <row r="416" ht="16" customHeight="1">
-      <c r="A416" s="12" t="inlineStr">
+      <c r="I416" s="16" t="inlineStr"/>
+    </row>
+    <row r="417" ht="16" customHeight="1">
+      <c r="A417" s="12" t="inlineStr">
         <is>
           <t>HU-69</t>
         </is>
       </c>
-      <c r="B416" s="12" t="inlineStr">
+      <c r="B417" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C416" s="12" t="inlineStr">
+      <c r="C417" s="12" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="D416" s="12" t="inlineStr">
+      <c r="D417" s="12" t="inlineStr">
         <is>
           <t>Como empleado quiero subir mi orden médica para justificar una ausencia.</t>
         </is>
       </c>
-      <c r="E416" s="13" t="inlineStr">
+      <c r="E417" s="13" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="F416" s="13" t="inlineStr">
+      <c r="F417" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G416" s="13" t="inlineStr">
+      <c r="G417" s="13" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H416" s="12" t="inlineStr">
+      <c r="H417" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I416" s="12" t="inlineStr"/>
-    </row>
-    <row r="417">
-      <c r="A417" s="14" t="inlineStr">
+      <c r="I417" s="12" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" s="14" t="inlineStr">
         <is>
           <t>T-69.1</t>
         </is>
       </c>
-      <c r="B417" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C417" s="14" t="inlineStr"/>
-      <c r="D417" s="14" t="inlineStr">
+      <c r="B418" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C418" s="14" t="inlineStr"/>
+      <c r="D418" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Definir el almacenamiento local de archivos adjuntos</t>
         </is>
       </c>
-      <c r="E417" s="15" t="inlineStr"/>
-      <c r="F417" s="15" t="inlineStr">
+      <c r="E418" s="15" t="inlineStr"/>
+      <c r="F418" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G417" s="15" t="inlineStr">
+      <c r="G418" s="15" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H417" s="14" t="inlineStr">
+      <c r="H418" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I417" s="14" t="inlineStr"/>
-    </row>
-    <row r="418">
-      <c r="A418" s="16" t="inlineStr">
+      <c r="I418" s="14" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" s="16" t="inlineStr">
         <is>
           <t>T-69.2</t>
         </is>
       </c>
-      <c r="B418" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C418" s="16" t="inlineStr"/>
-      <c r="D418" s="16" t="inlineStr">
+      <c r="B419" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C419" s="16" t="inlineStr"/>
+      <c r="D419" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar la subida con validación de tipo y tamaño</t>
         </is>
       </c>
-      <c r="E418" s="17" t="inlineStr"/>
-      <c r="F418" s="17" t="inlineStr">
+      <c r="E419" s="17" t="inlineStr"/>
+      <c r="F419" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G418" s="17" t="inlineStr">
+      <c r="G419" s="17" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H418" s="16" t="inlineStr">
+      <c r="H419" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I418" s="16" t="inlineStr"/>
-    </row>
-    <row r="419">
-      <c r="A419" s="14" t="inlineStr">
+      <c r="I419" s="16" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" s="14" t="inlineStr">
         <is>
           <t>T-69.3</t>
         </is>
       </c>
-      <c r="B419" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C419" s="14" t="inlineStr"/>
-      <c r="D419" s="14" t="inlineStr">
+      <c r="B420" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C420" s="14" t="inlineStr"/>
+      <c r="D420" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Restringir la visibilidad del archivo</t>
         </is>
       </c>
-      <c r="E419" s="15" t="inlineStr"/>
-      <c r="F419" s="15" t="inlineStr">
+      <c r="E420" s="15" t="inlineStr"/>
+      <c r="F420" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G419" s="15" t="inlineStr">
+      <c r="G420" s="15" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H419" s="14" t="inlineStr">
+      <c r="H420" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I419" s="14" t="inlineStr"/>
-    </row>
-    <row r="420">
-      <c r="A420" s="16" t="inlineStr">
+      <c r="I420" s="14" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" s="16" t="inlineStr">
         <is>
           <t>T-69.4</t>
         </is>
       </c>
-      <c r="B420" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C420" s="16" t="inlineStr"/>
-      <c r="D420" s="16" t="inlineStr">
+      <c r="B421" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C421" s="16" t="inlineStr"/>
+      <c r="D421" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Definir el tratamiento de los datos de salud</t>
         </is>
       </c>
-      <c r="E420" s="17" t="inlineStr"/>
-      <c r="F420" s="17" t="inlineStr">
+      <c r="E421" s="17" t="inlineStr"/>
+      <c r="F421" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G420" s="17" t="inlineStr">
+      <c r="G421" s="17" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H420" s="16" t="inlineStr">
+      <c r="H421" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I420" s="16" t="inlineStr"/>
-    </row>
-    <row r="421" ht="16" customHeight="1">
-      <c r="A421" s="12" t="inlineStr">
+      <c r="I421" s="16" t="inlineStr"/>
+    </row>
+    <row r="422" ht="16" customHeight="1">
+      <c r="A422" s="12" t="inlineStr">
         <is>
           <t>HU-70</t>
         </is>
       </c>
-      <c r="B421" s="12" t="inlineStr">
+      <c r="B422" s="12" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C421" s="12" t="inlineStr">
+      <c r="C422" s="12" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="D421" s="12" t="inlineStr">
+      <c r="D422" s="12" t="inlineStr">
         <is>
           <t>Como área de personal quiero ver el calendario de ausencias para organizar la cobertura.</t>
         </is>
       </c>
-      <c r="E421" s="13" t="inlineStr">
+      <c r="E422" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="F421" s="13" t="inlineStr">
+      <c r="F422" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G421" s="13" t="inlineStr">
+      <c r="G422" s="13" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H421" s="12" t="inlineStr">
+      <c r="H422" s="12" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I421" s="12" t="inlineStr"/>
-    </row>
-    <row r="422">
-      <c r="A422" s="14" t="inlineStr">
+      <c r="I422" s="12" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" s="14" t="inlineStr">
         <is>
           <t>T-70.1</t>
         </is>
       </c>
-      <c r="B422" s="14" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C422" s="14" t="inlineStr"/>
-      <c r="D422" s="14" t="inlineStr">
+      <c r="B423" s="14" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C423" s="14" t="inlineStr"/>
+      <c r="D423" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    Diseñar el calendario de ausencias</t>
         </is>
       </c>
-      <c r="E422" s="15" t="inlineStr"/>
-      <c r="F422" s="15" t="inlineStr">
+      <c r="E423" s="15" t="inlineStr"/>
+      <c r="F423" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G422" s="15" t="inlineStr">
+      <c r="G423" s="15" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H422" s="14" t="inlineStr">
+      <c r="H423" s="14" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I422" s="14" t="inlineStr"/>
-    </row>
-    <row r="423">
-      <c r="A423" s="16" t="inlineStr">
+      <c r="I423" s="14" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" s="16" t="inlineStr">
         <is>
           <t>T-70.2</t>
         </is>
       </c>
-      <c r="B423" s="16" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C423" s="16" t="inlineStr"/>
-      <c r="D423" s="16" t="inlineStr">
+      <c r="B424" s="16" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C424" s="16" t="inlineStr"/>
+      <c r="D424" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">    Programar la consulta por período</t>
         </is>
       </c>
-      <c r="E423" s="17" t="inlineStr"/>
-      <c r="F423" s="17" t="inlineStr">
+      <c r="E424" s="17" t="inlineStr"/>
+      <c r="F424" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G423" s="17" t="inlineStr">
+      <c r="G424" s="17" t="inlineStr">
         <is>
           <t>Sin asignar</t>
         </is>
       </c>
-      <c r="H423" s="16" t="inlineStr">
+      <c r="H424" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="I423" s="16" t="inlineStr"/>
+      <c r="I424" s="16" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I423"/>
+  <autoFilter ref="A4:I424"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H423">
+  <conditionalFormatting sqref="H5:H424">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Hecho"</formula>
     </cfRule>
@@ -23272,13 +23358,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H5:H423" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H424" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,En curso,En revisión,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E423" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E424" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja"</formula1>
     </dataValidation>
-    <dataValidation sqref="I5:I423" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I5:I424" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aguilera Maximiliano,Hoyos Franco,Delipetro Ezequiel,Achille Nahuel,Equipo"</formula1>
     </dataValidation>
   </dataValidations>
@@ -23593,7 +23679,7 @@
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cerrado</t>
         </is>
       </c>
     </row>
@@ -23630,7 +23716,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cerrado</t>
         </is>
       </c>
     </row>
@@ -23667,7 +23753,7 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cerrado</t>
         </is>
       </c>
     </row>
@@ -23704,7 +23790,7 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>Planificado</t>
+          <t>En curso</t>
         </is>
       </c>
     </row>
@@ -23741,7 +23827,7 @@
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>Planificado</t>
+          <t>En curso</t>
         </is>
       </c>
     </row>
@@ -23839,11 +23925,11 @@
         <v>7</v>
       </c>
       <c r="E17" s="15">
-        <f>SUMPRODUCT((LEFT('Sprint 13'!A6:A36,2)="T-")*1)</f>
+        <f>SUMPRODUCT((LEFT('Sprint 13'!A6:A37,2)="T-")*1)</f>
         <v/>
       </c>
       <c r="F17" s="15">
-        <f>SUMPRODUCT((LEFT('Sprint 13'!A6:A36,2)="T-")*('Sprint 13'!E6:E36="Hecho"))</f>
+        <f>SUMPRODUCT((LEFT('Sprint 13'!A6:A37,2)="T-")*('Sprint 13'!E6:E37="Hecho"))</f>
         <v/>
       </c>
       <c r="G17" s="18">
@@ -28041,7 +28127,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Período: 14/09 al 20/09    |    Estado: En curso</t>
+          <t>Período: 14/09 al 20/09    |    Estado: Cerrado</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>